<commit_message>
feat: add DEDI challenge and GENOVATE hackathon as submitted competitions in tracker and links.txt
</commit_message>
<xml_diff>
--- a/compitiations/Ally_Vision_Competitions_Master_Tracker_Updated.xlsx
+++ b/compitiations/Ally_Vision_Competitions_Master_Tracker_Updated.xlsx
@@ -22,7 +22,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="16">
+  <fonts count="17">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -104,6 +104,12 @@
     <font>
       <name val="Segoe UI"/>
       <b val="1"/>
+      <color rgb="003730A3"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Segoe UI"/>
+      <b val="1"/>
       <color rgb="001E293B"/>
       <sz val="11"/>
     </font>
@@ -120,7 +126,7 @@
       <sz val="9"/>
     </font>
   </fonts>
-  <fills count="12">
+  <fills count="13">
     <fill>
       <patternFill/>
     </fill>
@@ -179,6 +185,12 @@
       <patternFill patternType="solid">
         <fgColor rgb="00FEF3C7"/>
         <bgColor rgb="00FEF3C7"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E0E7FF"/>
+        <bgColor rgb="00E0E7FF"/>
       </patternFill>
     </fill>
     <fill>
@@ -258,7 +270,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="26">
+  <cellXfs count="27">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -309,20 +321,23 @@
     <xf numFmtId="0" fontId="12" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="13" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="15" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="16" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -2218,59 +2233,61 @@
       </c>
       <c r="B28" s="11" t="inlineStr">
         <is>
-          <t>برنامج إبتكار IbTIECar (جولة دعم التصنيع المتقدم)</t>
+          <t>تحدي DEDI للابتكار (DEDI Innovation Challenge)</t>
         </is>
       </c>
       <c r="C28" s="11" t="inlineStr">
         <is>
-          <t>مركز الإبداع التكنولوجي وريادة الأعمال (TIEC)</t>
+          <t>برنامج الأمم المتحدة الإنمائي (UNDP) &amp; CREATIVA &amp; ITIDA &amp; DEDI</t>
         </is>
       </c>
       <c r="D28" s="12" t="inlineStr">
         <is>
-          <t>https://tiec.gov.eg/Arabic/Programs/IBTIECAR/Pages/default.aspx</t>
+          <t>https://lnkd.in/p/eqgBp3t9</t>
         </is>
       </c>
       <c r="E28" s="13" t="inlineStr">
         <is>
-          <t>يناير 2027</t>
+          <t>أكتوبر 2026</t>
         </is>
       </c>
       <c r="F28" s="13" t="inlineStr">
         <is>
-          <t>الموعد النهائي: 28 فبراير 2027</t>
-        </is>
-      </c>
-      <c r="G28" s="17" t="inlineStr">
-        <is>
-          <t>لم تفتح بعد - متابعة (Pending)</t>
+          <t>الموعد النهائي: 27 أكتوبر 2026 (اليوم)</t>
+        </is>
+      </c>
+      <c r="G28" s="18" t="inlineStr">
+        <is>
+          <t>تم التقديم بنجاح (Submitted)</t>
         </is>
       </c>
       <c r="H28" s="11" t="inlineStr">
         <is>
-          <t>1. تقرير مرحلي عن النموذج الأولي (Progress Report Milestone)
-2. نتائج اختبارات المحاكاة والـ 3D Point Clouds
-3. مراجعة فواتير شراء المكونات</t>
+          <t>1. استمارة التقديم الرسمية
+2. وصف الفكرة وحل المشكلة المبتكر
+3. رابط النموذج الأولي والـ PoC على GitHub
+4. رابط نموذج العمل التجاري (BMC)
+5. بيانات برامج كرياتيفا السابقة وبيانات الفريق الـ 11</t>
         </is>
       </c>
       <c r="I28" s="11" t="inlineStr">
         <is>
-          <t>ICT Hardware / Software Acceleration</t>
+          <t>Social Impact &amp; Assistive DeepTech (UN SDGs 3 &amp; 10)</t>
         </is>
       </c>
       <c r="J28" s="11" t="inlineStr">
         <is>
-          <t>دعم تصنيع إضافي للمشاريع المتميزة واستشارات إرشادية وتأهيل للتأسيس القانوني للشركة</t>
-        </is>
-      </c>
-      <c r="K28" s="15" t="inlineStr">
-        <is>
-          <t>أولوية عالية (High)</t>
+          <t>شهادة معتمدة من الأمم المتحدة UNDP وكريتيفا + تأهيل مباشر لحاضنة أعمال متكاملة لتأسيس الشركة + تدريب وتوجيه تقني</t>
+        </is>
+      </c>
+      <c r="K28" s="9" t="inlineStr">
+        <is>
+          <t>أولوية قصوى (Very High)</t>
         </is>
       </c>
       <c r="L28" s="11" t="inlineStr">
         <is>
-          <t>متابعة دورية لتسليمات الدورة الأولى من إبتكار للمحافظة على موقع متميز في التصفيات المتقدمة.</t>
+          <t>تم التقديم بنجاح بالاستمارة الكاملة مع توفير روابط الـ BMC والـ PoC وبيانات الفريق المعتمدة.</t>
         </is>
       </c>
     </row>
@@ -2280,59 +2297,60 @@
       </c>
       <c r="B29" s="5" t="inlineStr">
         <is>
-          <t>برنامج إبتكار IbTIECar (معسكر التدريب الصيفي)</t>
+          <t>هاكاثون جينوفيت (GENOVATE HACKATHON)</t>
         </is>
       </c>
       <c r="C29" s="5" t="inlineStr">
         <is>
-          <t>مركز الإبداع التكنولوجي وريادة الأعمال (TIEC)</t>
+          <t>مراكز إبداع مصر الرقمية «كريتيفا إسكندرية» (Creativa Hub Alexandria)</t>
         </is>
       </c>
       <c r="D29" s="6" t="inlineStr">
         <is>
-          <t>https://tiec.gov.eg/Arabic/Programs/IBTIECAR/Pages/default.aspx</t>
+          <t>https://www.linkedin.com/posts/creativa-hub-alexandria_%D9%84%D9%88-%D8%B9%D9%86%D8%AF%D9%83-%D9%81%D9%83%D8%B1%D8%A9-%D8%AA%D8%BA%D9%8A%D8%B1-%D9%85%D8%B3%D8%AA%D9%82%D8%A8%D9%84-%D8%A7%D9%84%D8%AA%D8%B9%D9%84%D9%8A%D9%85-%D8%A3%D9%88-%D8%A7%D9%84%D8%B1%D8%B9%D8%A7%D9%8A%D8%A9-activity-7518280083271462912--CHD</t>
         </is>
       </c>
       <c r="E29" s="7" t="inlineStr">
         <is>
-          <t>مايو 2027</t>
+          <t>أكتوبر 2026</t>
         </is>
       </c>
       <c r="F29" s="7" t="inlineStr">
         <is>
-          <t>الموعد النهائي: 15 يونيو 2027</t>
-        </is>
-      </c>
-      <c r="G29" s="17" t="inlineStr">
-        <is>
-          <t>لم تفتح بعد - متابعة (Pending)</t>
+          <t>الموعد النهائي: أواخر أكتوبر 2026</t>
+        </is>
+      </c>
+      <c r="G29" s="18" t="inlineStr">
+        <is>
+          <t>تم التقديم بنجاح (Submitted)</t>
         </is>
       </c>
       <c r="H29" s="5" t="inlineStr">
         <is>
-          <t>1. النموذج الأولي الكامل المختبر مع مستخدمين حقيقيين
-2. الأطروحة الهندسية للمشروع (Graduation Thesis Draft)
-3. فيديو احترافي للحل النهائي</t>
+          <t>1. اختيار المسار (Health-Tech: التشخيص بالـ AI والرعاية الصحية)
+2. تشكيل فريق 3-5 أفراد (ممثلي الفريق)
+3. التحقق من احتياج السوق والـ Business Model وتطوير الـ MVP
+4. التحضير لعرض الـ Pitch أمام لجان التقييم</t>
         </is>
       </c>
       <c r="I29" s="5" t="inlineStr">
         <is>
-          <t>Startup Ready Prototypes Track</t>
+          <t>Health-Tech: AI &amp; Assistive Healthcare</t>
         </is>
       </c>
       <c r="J29" s="5" t="inlineStr">
         <is>
-          <t>فرصة الاحتضان المباشر في حاضنة Start-IT وتحويل المشروع مباشرة لشركة ناشئة بتمويل تأسيسي</t>
-        </is>
-      </c>
-      <c r="K29" s="15" t="inlineStr">
-        <is>
-          <t>أولوية عالية (High)</t>
+          <t>إجمالي جوائز 100,000 جنيه + Mentorship واستشارات متخصصة ومساحات عمل مشتركة وفرص للتواصل مع مستثمرين</t>
+        </is>
+      </c>
+      <c r="K29" s="9" t="inlineStr">
+        <is>
+          <t>أولوية قصوى (Very High)</t>
         </is>
       </c>
       <c r="L29" s="5" t="inlineStr">
         <is>
-          <t>مرحلة ما بعد مناقشة مشروع التخرج؛ نقلة نوعية من أروقة الجامعة إلى السوق التجاري مباشرة.</t>
+          <t>تم التقديم في مسار Health-Tech؛ الاستعداد لمرحلة معسكر التدريب وعرض الـ Pitch Deck أمام الحكام.</t>
         </is>
       </c>
     </row>
@@ -2856,7 +2874,7 @@
       </c>
     </row>
     <row r="5" ht="95" customHeight="1">
-      <c r="A5" s="18" t="inlineStr">
+      <c r="A5" s="19" t="inlineStr">
         <is>
           <t>ما هو عنوان وفكرة المشروع باختصار؟
 (Project Title &amp; Elevator Pitch)</t>
@@ -2877,7 +2895,7 @@
           <t>Ally Vision is a next-generation visual-to-tactile spatial navigation headset for the blind. It translates 3D environmental geometry into intuitive physical height profiles on the forehead using a 5x5 micro-pin actuator matrix and edge AI depth camera, delivering complete hands-free and ear-free mobility independence.</t>
         </is>
       </c>
-      <c r="E5" s="18" t="inlineStr">
+      <c r="E5" s="19" t="inlineStr">
         <is>
           <t>• 100% Ear-Free
 • 100% Hands-Free
@@ -2887,7 +2905,7 @@
       </c>
     </row>
     <row r="6" ht="95" customHeight="1">
-      <c r="A6" s="19" t="inlineStr">
+      <c r="A6" s="20" t="inlineStr">
         <is>
           <t>ما هي المشكلة المحددة التي يعالجها المشروع؟
 (The Problem Statement)</t>
@@ -2912,7 +2930,7 @@
 3. Existing high-tech European solutions (like 7Sense and BrainPort) cost $3,000 to $5,000+, putting them completely out of reach for users in developing markets.</t>
         </is>
       </c>
-      <c r="E6" s="19" t="inlineStr">
+      <c r="E6" s="20" t="inlineStr">
         <is>
           <t>• 285 مليون كفيف عالمياً
 • 1.5 مليون كفيف في مصر
@@ -2921,7 +2939,7 @@
       </c>
     </row>
     <row r="7" ht="95" customHeight="1">
-      <c r="A7" s="18" t="inlineStr">
+      <c r="A7" s="19" t="inlineStr">
         <is>
           <t>ما هو الحل والابتكار التقني الفريد؟
 (Solution &amp; Technical Innovation)</t>
@@ -2948,7 +2966,7 @@
 3. Output: 5x5 micro-actuator matrix modulating physical height displacement (levels 0-5) on the forehead, eliminating tactile sensory fatigue with &lt;100ms end-to-end latency.</t>
         </is>
       </c>
-      <c r="E7" s="18" t="inlineStr">
+      <c r="E7" s="19" t="inlineStr">
         <is>
           <t>• RANSAC Ground Clearance
 • ByteTrack Velocity (dZ/dt)
@@ -2958,7 +2976,7 @@
       </c>
     </row>
     <row r="8" ht="95" customHeight="1">
-      <c r="A8" s="19" t="inlineStr">
+      <c r="A8" s="20" t="inlineStr">
         <is>
           <t>من هي الشريحة المستهدفة وما حجم السوق؟
 (Target Market &amp; Customer Segments)</t>
@@ -2985,7 +3003,7 @@
 • Target Segments: Active visually impaired students and professionals (B2C), Blind Welfare NGOs and rehabilitation hubs (B2G/B2B), and Corporate Social Responsibility (CSR) donors.</t>
         </is>
       </c>
-      <c r="E8" s="19" t="inlineStr">
+      <c r="E8" s="20" t="inlineStr">
         <is>
           <t>• TAM: $31.4B
 • SAM: 40M+
@@ -2995,7 +3013,7 @@
       </c>
     </row>
     <row r="9" ht="95" customHeight="1">
-      <c r="A9" s="18" t="inlineStr">
+      <c r="A9" s="19" t="inlineStr">
         <is>
           <t>ما هي الميزة التنافسية؟ ولماذا يتفوق مشروعكم؟
 (Competitive Advantage &amp; Moat)</t>
@@ -3022,7 +3040,7 @@
 4. Frugal Engineering: Custom BOM and PCB architecture lowering production cost to &lt;20% of Western competitors (retail target &lt;$400 vs $4,000+).</t>
         </is>
       </c>
-      <c r="E9" s="18" t="inlineStr">
+      <c r="E9" s="19" t="inlineStr">
         <is>
           <t>• تكلفة &lt; 20% من 7Sense
 • تفادي خدر الجلد (No Sensory Fatigue)
@@ -3031,7 +3049,7 @@
       </c>
     </row>
     <row r="10" ht="95" customHeight="1">
-      <c r="A10" s="19" t="inlineStr">
+      <c r="A10" s="20" t="inlineStr">
         <is>
           <t>ما هو نموذج العمل وتوليد الإيرادات؟
 (Business Model &amp; Revenue Streams)</t>
@@ -3058,7 +3076,7 @@
 4. Hardware-as-a-Service (HaaS): Optional annual subscription for mechanical pin maintenance, warranty, and over-the-air AI upgrades.</t>
         </is>
       </c>
-      <c r="E10" s="19" t="inlineStr">
+      <c r="E10" s="20" t="inlineStr">
         <is>
           <t>• B2B2C Framework
 • CSR Funding Contracts
@@ -3068,7 +3086,7 @@
       </c>
     </row>
     <row r="11" ht="95" customHeight="1">
-      <c r="A11" s="18" t="inlineStr">
+      <c r="A11" s="19" t="inlineStr">
         <is>
           <t>ما هي المرحلة الحالية للمشروع وما الذي تم إنجازه؟
 (Current Traction &amp; Milestones)</t>
@@ -3095,7 +3113,7 @@
 4. Curated a custom 2,000-image navigation dataset and synthesized 137 academic papers on sensory substitution and tactile neuroscience.</t>
         </is>
       </c>
-      <c r="E11" s="18" t="inlineStr">
+      <c r="E11" s="19" t="inlineStr">
         <is>
           <t>• 2,000 Annotated Images
 • sub-20ms AI Inference
@@ -3105,7 +3123,7 @@
       </c>
     </row>
     <row r="12" ht="95" customHeight="1">
-      <c r="A12" s="19" t="inlineStr">
+      <c r="A12" s="20" t="inlineStr">
         <is>
           <t>ما هي احتياجات المعامل والدعم الفني المطلوب؟
 (FabLab &amp; IoT Lab Support Needs)</t>
@@ -3130,7 +3148,7 @@
 3. Mentorship Needs: Guidance on hardware miniaturization, battery power management, ergonomic compliance, and intellectual property (IP) filing.</t>
         </is>
       </c>
-      <c r="E12" s="19" t="inlineStr">
+      <c r="E12" s="20" t="inlineStr">
         <is>
           <t>• 3D Printing (Visor Enclosure)
 • Custom Multi-layer PCB Milling
@@ -3180,14 +3198,14 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="20" t="inlineStr">
+      <c r="A4" s="21" t="inlineStr">
         <is>
           <t>بيانات المؤسسة والمشروع الأكاديمي</t>
         </is>
       </c>
     </row>
     <row r="5" ht="22" customHeight="1">
-      <c r="A5" s="19" t="inlineStr">
+      <c r="A5" s="20" t="inlineStr">
         <is>
           <t>الجامعة (University)</t>
         </is>
@@ -3197,12 +3215,12 @@
           <t>الجامعة المصرية الصينية - Egyptian Chinese University (ECU)</t>
         </is>
       </c>
-      <c r="C5" s="21" t="n"/>
-      <c r="D5" s="21" t="n"/>
-      <c r="E5" s="22" t="n"/>
+      <c r="C5" s="22" t="n"/>
+      <c r="D5" s="22" t="n"/>
+      <c r="E5" s="23" t="n"/>
     </row>
     <row r="6" ht="22" customHeight="1">
-      <c r="A6" s="19" t="inlineStr">
+      <c r="A6" s="20" t="inlineStr">
         <is>
           <t>الكلية (College / Faculty)</t>
         </is>
@@ -3212,12 +3230,12 @@
           <t>كلية الهندسة والتكنولوجيا - Faculty of Engineering and Technology</t>
         </is>
       </c>
-      <c r="C6" s="21" t="n"/>
-      <c r="D6" s="21" t="n"/>
-      <c r="E6" s="22" t="n"/>
+      <c r="C6" s="22" t="n"/>
+      <c r="D6" s="22" t="n"/>
+      <c r="E6" s="23" t="n"/>
     </row>
     <row r="7" ht="22" customHeight="1">
-      <c r="A7" s="19" t="inlineStr">
+      <c r="A7" s="20" t="inlineStr">
         <is>
           <t>المشرف الأكاديمي (Academic Supervisor)</t>
         </is>
@@ -3227,12 +3245,12 @@
           <t>د. إسلام محمد (Dr. Islam Mohamed)</t>
         </is>
       </c>
-      <c r="C7" s="21" t="n"/>
-      <c r="D7" s="21" t="n"/>
-      <c r="E7" s="22" t="n"/>
+      <c r="C7" s="22" t="n"/>
+      <c r="D7" s="22" t="n"/>
+      <c r="E7" s="23" t="n"/>
     </row>
     <row r="8" ht="22" customHeight="1">
-      <c r="A8" s="19" t="inlineStr">
+      <c r="A8" s="20" t="inlineStr">
         <is>
           <t>عنوان المشروع الرسمي (Official Title)</t>
         </is>
@@ -3242,12 +3260,12 @@
           <t>Ally Vision: AI-Powered Assistive Vision &amp; Navigation System for the Blind</t>
         </is>
       </c>
-      <c r="C8" s="21" t="n"/>
-      <c r="D8" s="21" t="n"/>
-      <c r="E8" s="22" t="n"/>
+      <c r="C8" s="22" t="n"/>
+      <c r="D8" s="22" t="n"/>
+      <c r="E8" s="23" t="n"/>
     </row>
     <row r="9" ht="22" customHeight="1">
-      <c r="A9" s="19" t="inlineStr">
+      <c r="A9" s="20" t="inlineStr">
         <is>
           <t>المجال التقني (Domain)</t>
         </is>
@@ -3257,12 +3275,12 @@
           <t>الذكاء الاصطناعي، الروبوتات، التكنولوجيا المساعدة، والأنظمة المدمجة (AI, Robotics &amp; Assistive Tech)</t>
         </is>
       </c>
-      <c r="C9" s="21" t="n"/>
-      <c r="D9" s="21" t="n"/>
-      <c r="E9" s="22" t="n"/>
+      <c r="C9" s="22" t="n"/>
+      <c r="D9" s="22" t="n"/>
+      <c r="E9" s="23" t="n"/>
     </row>
     <row r="10" ht="22" customHeight="1">
-      <c r="A10" s="19" t="inlineStr">
+      <c r="A10" s="20" t="inlineStr">
         <is>
           <t>المرحلة الحالية (Current Stage)</t>
         </is>
@@ -3272,12 +3290,12 @@
           <t>نموذج أولي متقدم ومختبر برمجياً (Advanced Working Prototype &amp; Simulation)</t>
         </is>
       </c>
-      <c r="C10" s="21" t="n"/>
-      <c r="D10" s="21" t="n"/>
-      <c r="E10" s="22" t="n"/>
+      <c r="C10" s="22" t="n"/>
+      <c r="D10" s="22" t="n"/>
+      <c r="E10" s="23" t="n"/>
     </row>
     <row r="11" ht="22" customHeight="1">
-      <c r="A11" s="19" t="inlineStr">
+      <c r="A11" s="20" t="inlineStr">
         <is>
           <t>حجم الفريق (Team Size)</t>
         </is>
@@ -3287,12 +3305,12 @@
           <t>11 مهندساً (Multidisciplinary Engineering Team)</t>
         </is>
       </c>
-      <c r="C11" s="21" t="n"/>
-      <c r="D11" s="21" t="n"/>
-      <c r="E11" s="22" t="n"/>
+      <c r="C11" s="22" t="n"/>
+      <c r="D11" s="22" t="n"/>
+      <c r="E11" s="23" t="n"/>
     </row>
     <row r="12" ht="22" customHeight="1">
-      <c r="A12" s="19" t="inlineStr">
+      <c r="A12" s="20" t="inlineStr">
         <is>
           <t>رابط مجلد الملفات (Google Drive Folder)</t>
         </is>
@@ -3302,12 +3320,12 @@
           <t>https://drive.google.com/drive/folders/ally-vision-ecu (يحوي البطاقات، السير الذاتية، المقترح، والـ Deck)</t>
         </is>
       </c>
-      <c r="C12" s="21" t="n"/>
-      <c r="D12" s="21" t="n"/>
-      <c r="E12" s="22" t="n"/>
+      <c r="C12" s="22" t="n"/>
+      <c r="D12" s="22" t="n"/>
+      <c r="E12" s="23" t="n"/>
     </row>
     <row r="14">
-      <c r="A14" s="20" t="inlineStr">
+      <c r="A14" s="21" t="inlineStr">
         <is>
           <t>قائمة أعضاء الفريق (11 مهندساً)</t>
         </is>
@@ -3736,39 +3754,39 @@
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="20" t="inlineStr">
+      <c r="A28" s="21" t="inlineStr">
         <is>
           <t>جدول الميزانية التقديرية المطلوبة للمشروع (Budget Breakdown)</t>
         </is>
       </c>
     </row>
     <row r="29" ht="26" customHeight="1">
-      <c r="A29" s="23" t="inlineStr">
+      <c r="A29" s="24" t="inlineStr">
         <is>
           <t>بند الميزانية (Category)</t>
         </is>
       </c>
-      <c r="B29" s="23" t="inlineStr">
+      <c r="B29" s="24" t="inlineStr">
         <is>
           <t>المكونات والمواصفات التفصيلية</t>
         </is>
       </c>
-      <c r="C29" s="23" t="inlineStr">
+      <c r="C29" s="24" t="inlineStr">
         <is>
           <t>الكمية</t>
         </is>
       </c>
-      <c r="D29" s="23" t="inlineStr">
+      <c r="D29" s="24" t="inlineStr">
         <is>
           <t>التكلفة بالجنيه المصري (EGP)</t>
         </is>
       </c>
-      <c r="E29" s="23" t="inlineStr">
+      <c r="E29" s="24" t="inlineStr">
         <is>
           <t>النسبة من الميزانية</t>
         </is>
       </c>
-      <c r="F29" s="23" t="inlineStr">
+      <c r="F29" s="24" t="inlineStr">
         <is>
           <t>الأهمية والأثر الهندسي</t>
         </is>
@@ -3935,13 +3953,13 @@
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="24" t="inlineStr">
+      <c r="A35" s="25" t="inlineStr">
         <is>
           <t>إجمالي الميزانية المطلوبة (Total Required Budget)</t>
         </is>
       </c>
-      <c r="B35" s="21" t="n"/>
-      <c r="C35" s="22" t="n"/>
+      <c r="B35" s="22" t="n"/>
+      <c r="C35" s="23" t="n"/>
       <c r="D35" s="3" t="inlineStr">
         <is>
           <t>85,000 ج (~ $1,750)</t>
@@ -3952,7 +3970,7 @@
           <t>100%</t>
         </is>
       </c>
-      <c r="F35" s="25" t="inlineStr">
+      <c r="F35" s="26" t="inlineStr">
         <is>
           <t>ميزانية نموذج أولي كامل جاهز للاختبارات السريرية الميدانية</t>
         </is>

</xml_diff>